<commit_message>
Update notebook - missing values
</commit_message>
<xml_diff>
--- a/data/ML_project_kidney_disease.xlsx
+++ b/data/ML_project_kidney_disease.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RhondaSwider\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RhondaSwider\Downloads\ISDS7075\Chronic Kidney Disease\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEF18766-1B3E-4782-B80D-F239B4F0CDEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E86536CD-3BA9-4FCA-85AD-DD20A03225B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1170" yWindow="1170" windowWidth="13635" windowHeight="11295" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ML_project_kidney_disease" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4307" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4307" uniqueCount="101">
   <si>
     <t>id</t>
   </si>
@@ -191,9 +191,6 @@
     <t>blood gluucose random</t>
   </si>
   <si>
-    <t>buu</t>
-  </si>
-  <si>
     <t>blood urea</t>
   </si>
   <si>
@@ -255,9 +252,6 @@
   </si>
   <si>
     <t>chronic  kidney disease  class</t>
-  </si>
-  <si>
-    <t>var_info</t>
   </si>
   <si>
     <t>age in years</t>
@@ -327,6 +321,9 @@
   </si>
   <si>
     <t>class - (1,0)</t>
+  </si>
+  <si>
+    <t>value_info</t>
   </si>
 </sst>
 </file>
@@ -940,6 +937,7 @@
     <xf numFmtId="0" fontId="0" fillId="34" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="35" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="36" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -949,7 +947,6 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1398,10 +1395,10 @@
       <c r="AA1" t="s">
         <v>26</v>
       </c>
-      <c r="AI1" s="13"/>
-      <c r="AJ1" s="14"/>
-      <c r="AK1" s="14"/>
-      <c r="AL1" s="15"/>
+      <c r="AI1" s="14"/>
+      <c r="AJ1" s="15"/>
+      <c r="AK1" s="15"/>
+      <c r="AL1" s="16"/>
     </row>
     <row r="2" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A2" s="4">
@@ -31601,20 +31598,21 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="22.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="26.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="13" t="s">
         <v>45</v>
       </c>
-      <c r="B1" s="16" t="s">
+      <c r="B1" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="C1" s="16" t="s">
-        <v>72</v>
-      </c>
-      <c r="D1" s="16" t="s">
-        <v>78</v>
+      <c r="C1" s="13" t="s">
+        <v>71</v>
+      </c>
+      <c r="D1" s="13" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -31625,10 +31623,10 @@
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D2" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -31639,10 +31637,10 @@
         <v>47</v>
       </c>
       <c r="C3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D3" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -31653,10 +31651,10 @@
         <v>48</v>
       </c>
       <c r="C4" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D4" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -31667,10 +31665,10 @@
         <v>49</v>
       </c>
       <c r="C5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D5" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -31681,10 +31679,10 @@
         <v>50</v>
       </c>
       <c r="C6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D6" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -31695,10 +31693,10 @@
         <v>51</v>
       </c>
       <c r="C7" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D7" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -31709,10 +31707,10 @@
         <v>52</v>
       </c>
       <c r="C8" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D8" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -31723,10 +31721,10 @@
         <v>53</v>
       </c>
       <c r="C9" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D9" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -31737,10 +31735,10 @@
         <v>54</v>
       </c>
       <c r="C10" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D10" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
@@ -31751,24 +31749,24 @@
         <v>55</v>
       </c>
       <c r="C11" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D11" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
         <v>56</v>
       </c>
-      <c r="B12" t="s">
-        <v>57</v>
-      </c>
       <c r="C12" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
@@ -31776,13 +31774,13 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C13" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D13" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
@@ -31790,13 +31788,13 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C14" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D14" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
@@ -31804,13 +31802,13 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C15" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D15" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
@@ -31818,13 +31816,13 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C16" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D16" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
@@ -31832,13 +31830,13 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C17" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D17" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
@@ -31846,13 +31844,13 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C18" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D18" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
@@ -31860,13 +31858,13 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C19" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D19" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
@@ -31874,13 +31872,13 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C20" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D20" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
@@ -31888,13 +31886,13 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C21" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D21" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
@@ -31902,13 +31900,13 @@
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C22" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D22" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
@@ -31916,13 +31914,13 @@
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C23" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D23" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
@@ -31930,13 +31928,13 @@
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C24" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D24" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
@@ -31944,27 +31942,27 @@
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C25" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D25" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B26" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C26" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D26" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
@@ -31972,13 +31970,13 @@
         <v>26</v>
       </c>
       <c r="B27" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C27" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D27" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
     </row>
   </sheetData>

</xml_diff>